<commit_message>
Did all the data cleaning
</commit_message>
<xml_diff>
--- a/5_documentation/actSpgaAGJmEJWoGmeU4Fz.xlsx
+++ b/5_documentation/actSpgaAGJmEJWoGmeU4Fz.xlsx
@@ -1,11 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30502"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="124226"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{64EF9FD0-9F4A-4713-AA91-F5CDE0926700}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://samriddhitpf-my.sharepoint.com/personal/arpan_samriddhi_org/Documents/Projects/FNF/5_documentation/"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="2" documentId="8_{64EF9FD0-9F4A-4713-AA91-F5CDE0926700}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7A5D3563-9EF3-41B1-97B3-CC0FF7042E7D}"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView minimized="1" xWindow="380" yWindow="380" windowWidth="14400" windowHeight="8170" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="survey" sheetId="1" r:id="rId1"/>
@@ -2442,7 +2447,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1">
+  <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -2778,21 +2783,21 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:K142"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="26.140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="26.1796875" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="41" bestFit="1" customWidth="1"/>
-    <col min="3" max="4" width="255.7109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="4" width="255.7265625" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="32" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="30.28515625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="8.5703125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="53.85546875" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="17.140625" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="30.5703125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="30.26953125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="8.54296875" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="53.81640625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="17.1796875" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="30.54296875" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="30" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -2827,7 +2832,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="2" spans="1:11">
+    <row r="2" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>11</v>
       </c>
@@ -2844,7 +2849,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="3" spans="1:11">
+    <row r="3" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>16</v>
       </c>
@@ -2861,7 +2866,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="4" spans="1:11">
+    <row r="4" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>20</v>
       </c>
@@ -2878,12 +2883,12 @@
         <v>24</v>
       </c>
     </row>
-    <row r="5" spans="1:11">
+    <row r="5" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="6" spans="1:11">
+    <row r="6" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>26</v>
       </c>
@@ -2903,7 +2908,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="7" spans="1:11">
+    <row r="7" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>11</v>
       </c>
@@ -2923,7 +2928,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="8" spans="1:11">
+    <row r="8" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>16</v>
       </c>
@@ -2940,7 +2945,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="9" spans="1:11">
+    <row r="9" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>38</v>
       </c>
@@ -2957,7 +2962,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="10" spans="1:11">
+    <row r="10" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>42</v>
       </c>
@@ -2974,7 +2979,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="11" spans="1:11">
+    <row r="11" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>46</v>
       </c>
@@ -2991,7 +2996,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="12" spans="1:11">
+    <row r="12" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>50</v>
       </c>
@@ -3008,7 +3013,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="13" spans="1:11">
+    <row r="13" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>53</v>
       </c>
@@ -3025,7 +3030,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="14" spans="1:11">
+    <row r="14" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
         <v>53</v>
       </c>
@@ -3042,7 +3047,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="15" spans="1:11">
+    <row r="15" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
         <v>16</v>
       </c>
@@ -3059,7 +3064,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="16" spans="1:11">
+    <row r="16" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
         <v>16</v>
       </c>
@@ -3076,7 +3081,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="17" spans="1:11">
+    <row r="17" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
         <v>66</v>
       </c>
@@ -3102,7 +3107,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="18" spans="1:11">
+    <row r="18" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
         <v>73</v>
       </c>
@@ -3119,7 +3124,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="19" spans="1:11">
+    <row r="19" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
         <v>53</v>
       </c>
@@ -3139,7 +3144,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="20" spans="1:11">
+    <row r="20" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
         <v>81</v>
       </c>
@@ -3156,7 +3161,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="21" spans="1:11">
+    <row r="21" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
         <v>85</v>
       </c>
@@ -3176,7 +3181,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="22" spans="1:11">
+    <row r="22" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
         <v>85</v>
       </c>
@@ -3196,7 +3201,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="23" spans="1:11">
+    <row r="23" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
         <v>85</v>
       </c>
@@ -3216,7 +3221,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="24" spans="1:11">
+    <row r="24" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
         <v>85</v>
       </c>
@@ -3236,7 +3241,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="25" spans="1:11">
+    <row r="25" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
         <v>101</v>
       </c>
@@ -3253,7 +3258,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="26" spans="1:11">
+    <row r="26" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A26" t="s">
         <v>105</v>
       </c>
@@ -3270,7 +3275,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="27" spans="1:11">
+    <row r="27" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A27" t="s">
         <v>109</v>
       </c>
@@ -3290,7 +3295,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="28" spans="1:11">
+    <row r="28" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A28" t="s">
         <v>114</v>
       </c>
@@ -3307,7 +3312,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="29" spans="1:11">
+    <row r="29" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A29" t="s">
         <v>118</v>
       </c>
@@ -3324,7 +3329,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="30" spans="1:11">
+    <row r="30" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A30" t="s">
         <v>122</v>
       </c>
@@ -3341,7 +3346,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="31" spans="1:11">
+    <row r="31" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A31" t="s">
         <v>126</v>
       </c>
@@ -3364,7 +3369,7 @@
         <v>131</v>
       </c>
     </row>
-    <row r="32" spans="1:11">
+    <row r="32" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A32" t="s">
         <v>132</v>
       </c>
@@ -3381,7 +3386,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="33" spans="1:8">
+    <row r="33" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A33" t="s">
         <v>136</v>
       </c>
@@ -3407,7 +3412,7 @@
         <v>142</v>
       </c>
     </row>
-    <row r="34" spans="1:8">
+    <row r="34" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A34" t="s">
         <v>143</v>
       </c>
@@ -3433,7 +3438,7 @@
         <v>149</v>
       </c>
     </row>
-    <row r="35" spans="1:8">
+    <row r="35" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A35" t="s">
         <v>16</v>
       </c>
@@ -3450,7 +3455,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="36" spans="1:8">
+    <row r="36" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A36" t="s">
         <v>16</v>
       </c>
@@ -3467,7 +3472,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="37" spans="1:8">
+    <row r="37" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A37" t="s">
         <v>156</v>
       </c>
@@ -3484,7 +3489,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="38" spans="1:8">
+    <row r="38" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A38" t="s">
         <v>160</v>
       </c>
@@ -3501,7 +3506,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="39" spans="1:8">
+    <row r="39" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A39" t="s">
         <v>122</v>
       </c>
@@ -3518,7 +3523,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="40" spans="1:8">
+    <row r="40" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A40" t="s">
         <v>167</v>
       </c>
@@ -3538,7 +3543,7 @@
         <v>171</v>
       </c>
     </row>
-    <row r="41" spans="1:8">
+    <row r="41" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A41" t="s">
         <v>172</v>
       </c>
@@ -3558,7 +3563,7 @@
         <v>176</v>
       </c>
     </row>
-    <row r="42" spans="1:8">
+    <row r="42" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A42" t="s">
         <v>53</v>
       </c>
@@ -3578,7 +3583,7 @@
         <v>180</v>
       </c>
     </row>
-    <row r="43" spans="1:8">
+    <row r="43" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A43" t="s">
         <v>167</v>
       </c>
@@ -3598,7 +3603,7 @@
         <v>184</v>
       </c>
     </row>
-    <row r="44" spans="1:8">
+    <row r="44" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A44" t="s">
         <v>172</v>
       </c>
@@ -3618,7 +3623,7 @@
         <v>188</v>
       </c>
     </row>
-    <row r="45" spans="1:8">
+    <row r="45" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A45" t="s">
         <v>53</v>
       </c>
@@ -3638,7 +3643,7 @@
         <v>191</v>
       </c>
     </row>
-    <row r="46" spans="1:8">
+    <row r="46" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A46" t="s">
         <v>167</v>
       </c>
@@ -3658,7 +3663,7 @@
         <v>171</v>
       </c>
     </row>
-    <row r="47" spans="1:8">
+    <row r="47" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A47" t="s">
         <v>172</v>
       </c>
@@ -3678,7 +3683,7 @@
         <v>198</v>
       </c>
     </row>
-    <row r="48" spans="1:8">
+    <row r="48" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A48" t="s">
         <v>53</v>
       </c>
@@ -3698,7 +3703,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="49" spans="1:8">
+    <row r="49" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A49" t="s">
         <v>16</v>
       </c>
@@ -3715,7 +3720,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="50" spans="1:8">
+    <row r="50" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A50" t="s">
         <v>204</v>
       </c>
@@ -3732,7 +3737,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="51" spans="1:8">
+    <row r="51" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A51" t="s">
         <v>208</v>
       </c>
@@ -3752,7 +3757,7 @@
         <v>212</v>
       </c>
     </row>
-    <row r="52" spans="1:8">
+    <row r="52" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A52" t="s">
         <v>16</v>
       </c>
@@ -3769,7 +3774,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="53" spans="1:8">
+    <row r="53" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A53" t="s">
         <v>16</v>
       </c>
@@ -3792,7 +3797,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="54" spans="1:8">
+    <row r="54" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A54" t="s">
         <v>221</v>
       </c>
@@ -3809,7 +3814,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="55" spans="1:8">
+    <row r="55" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A55" t="s">
         <v>221</v>
       </c>
@@ -3826,7 +3831,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="56" spans="1:8">
+    <row r="56" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A56" t="s">
         <v>221</v>
       </c>
@@ -3843,7 +3848,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="57" spans="1:8">
+    <row r="57" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A57" t="s">
         <v>221</v>
       </c>
@@ -3860,7 +3865,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="58" spans="1:8">
+    <row r="58" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A58" t="s">
         <v>221</v>
       </c>
@@ -3877,7 +3882,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="59" spans="1:8">
+    <row r="59" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A59" t="s">
         <v>221</v>
       </c>
@@ -3894,7 +3899,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="60" spans="1:8">
+    <row r="60" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A60" t="s">
         <v>240</v>
       </c>
@@ -3911,7 +3916,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="61" spans="1:8">
+    <row r="61" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A61" t="s">
         <v>16</v>
       </c>
@@ -3928,7 +3933,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="62" spans="1:8">
+    <row r="62" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A62" t="s">
         <v>16</v>
       </c>
@@ -3945,7 +3950,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="63" spans="1:8">
+    <row r="63" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A63" t="s">
         <v>156</v>
       </c>
@@ -3962,7 +3967,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="64" spans="1:8">
+    <row r="64" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A64" t="s">
         <v>156</v>
       </c>
@@ -3979,7 +3984,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="65" spans="1:7">
+    <row r="65" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A65" t="s">
         <v>256</v>
       </c>
@@ -3996,7 +4001,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="66" spans="1:7">
+    <row r="66" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A66" t="s">
         <v>156</v>
       </c>
@@ -4013,7 +4018,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="67" spans="1:7">
+    <row r="67" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A67" t="s">
         <v>263</v>
       </c>
@@ -4030,7 +4035,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="68" spans="1:7">
+    <row r="68" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A68" t="s">
         <v>156</v>
       </c>
@@ -4047,7 +4052,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="69" spans="1:7">
+    <row r="69" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A69" t="s">
         <v>156</v>
       </c>
@@ -4064,7 +4069,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="70" spans="1:7">
+    <row r="70" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A70" t="s">
         <v>156</v>
       </c>
@@ -4081,7 +4086,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="71" spans="1:7">
+    <row r="71" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A71" t="s">
         <v>156</v>
       </c>
@@ -4098,7 +4103,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="72" spans="1:7">
+    <row r="72" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A72" t="s">
         <v>279</v>
       </c>
@@ -4115,7 +4120,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="73" spans="1:7">
+    <row r="73" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A73" t="s">
         <v>283</v>
       </c>
@@ -4132,7 +4137,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="74" spans="1:7">
+    <row r="74" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A74" t="s">
         <v>283</v>
       </c>
@@ -4149,7 +4154,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="75" spans="1:7">
+    <row r="75" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A75" t="s">
         <v>283</v>
       </c>
@@ -4166,7 +4171,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="76" spans="1:7">
+    <row r="76" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A76" t="s">
         <v>16</v>
       </c>
@@ -4183,7 +4188,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="77" spans="1:7">
+    <row r="77" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A77" t="s">
         <v>296</v>
       </c>
@@ -4200,7 +4205,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="78" spans="1:7">
+    <row r="78" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A78" t="s">
         <v>296</v>
       </c>
@@ -4217,7 +4222,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="79" spans="1:7">
+    <row r="79" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A79" t="s">
         <v>296</v>
       </c>
@@ -4234,7 +4239,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="80" spans="1:7">
+    <row r="80" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A80" t="s">
         <v>296</v>
       </c>
@@ -4251,7 +4256,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="81" spans="1:7">
+    <row r="81" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A81" t="s">
         <v>16</v>
       </c>
@@ -4268,7 +4273,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="82" spans="1:7">
+    <row r="82" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A82" t="s">
         <v>156</v>
       </c>
@@ -4285,7 +4290,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="83" spans="1:7">
+    <row r="83" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A83" t="s">
         <v>315</v>
       </c>
@@ -4302,7 +4307,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="84" spans="1:7">
+    <row r="84" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A84" t="s">
         <v>156</v>
       </c>
@@ -4319,7 +4324,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="85" spans="1:7">
+    <row r="85" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A85" t="s">
         <v>156</v>
       </c>
@@ -4336,7 +4341,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="86" spans="1:7">
+    <row r="86" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A86" t="s">
         <v>156</v>
       </c>
@@ -4353,7 +4358,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="87" spans="1:7">
+    <row r="87" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A87" t="s">
         <v>156</v>
       </c>
@@ -4370,7 +4375,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="88" spans="1:7">
+    <row r="88" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A88" t="s">
         <v>156</v>
       </c>
@@ -4387,7 +4392,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="89" spans="1:7">
+    <row r="89" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A89" t="s">
         <v>156</v>
       </c>
@@ -4404,7 +4409,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="90" spans="1:7">
+    <row r="90" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A90" t="s">
         <v>16</v>
       </c>
@@ -4421,7 +4426,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="91" spans="1:7">
+    <row r="91" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A91" t="s">
         <v>156</v>
       </c>
@@ -4438,7 +4443,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="92" spans="1:7">
+    <row r="92" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A92" t="s">
         <v>156</v>
       </c>
@@ -4455,7 +4460,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="93" spans="1:7">
+    <row r="93" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A93" t="s">
         <v>156</v>
       </c>
@@ -4472,7 +4477,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="94" spans="1:7">
+    <row r="94" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A94" t="s">
         <v>156</v>
       </c>
@@ -4489,7 +4494,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="95" spans="1:7">
+    <row r="95" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A95" t="s">
         <v>16</v>
       </c>
@@ -4506,7 +4511,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="96" spans="1:7">
+    <row r="96" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A96" t="s">
         <v>16</v>
       </c>
@@ -4523,7 +4528,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="97" spans="1:7">
+    <row r="97" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A97" t="s">
         <v>358</v>
       </c>
@@ -4540,7 +4545,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="98" spans="1:7">
+    <row r="98" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A98" t="s">
         <v>16</v>
       </c>
@@ -4557,7 +4562,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="99" spans="1:7">
+    <row r="99" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A99" t="s">
         <v>156</v>
       </c>
@@ -4574,7 +4579,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="100" spans="1:7">
+    <row r="100" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A100" t="s">
         <v>156</v>
       </c>
@@ -4591,7 +4596,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="101" spans="1:7">
+    <row r="101" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A101" t="s">
         <v>156</v>
       </c>
@@ -4608,7 +4613,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="102" spans="1:7">
+    <row r="102" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A102" t="s">
         <v>156</v>
       </c>
@@ -4625,7 +4630,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="103" spans="1:7">
+    <row r="103" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A103" t="s">
         <v>156</v>
       </c>
@@ -4642,7 +4647,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="104" spans="1:7">
+    <row r="104" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A104" t="s">
         <v>156</v>
       </c>
@@ -4659,7 +4664,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="105" spans="1:7">
+    <row r="105" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A105" t="s">
         <v>156</v>
       </c>
@@ -4676,7 +4681,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="106" spans="1:7">
+    <row r="106" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A106" t="s">
         <v>156</v>
       </c>
@@ -4693,7 +4698,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="107" spans="1:7">
+    <row r="107" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A107" t="s">
         <v>156</v>
       </c>
@@ -4710,7 +4715,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="108" spans="1:7">
+    <row r="108" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A108" t="s">
         <v>156</v>
       </c>
@@ -4727,7 +4732,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="109" spans="1:7">
+    <row r="109" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A109" t="s">
         <v>156</v>
       </c>
@@ -4744,7 +4749,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="110" spans="1:7">
+    <row r="110" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A110" t="s">
         <v>156</v>
       </c>
@@ -4761,7 +4766,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="111" spans="1:7">
+    <row r="111" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A111" t="s">
         <v>156</v>
       </c>
@@ -4778,7 +4783,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="112" spans="1:7">
+    <row r="112" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A112" t="s">
         <v>156</v>
       </c>
@@ -4795,7 +4800,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="113" spans="1:7">
+    <row r="113" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A113" t="s">
         <v>16</v>
       </c>
@@ -4812,7 +4817,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="114" spans="1:7">
+    <row r="114" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A114" t="s">
         <v>16</v>
       </c>
@@ -4829,7 +4834,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="115" spans="1:7">
+    <row r="115" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A115" t="s">
         <v>413</v>
       </c>
@@ -4846,7 +4851,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="116" spans="1:7">
+    <row r="116" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A116" t="s">
         <v>16</v>
       </c>
@@ -4863,7 +4868,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="117" spans="1:7">
+    <row r="117" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A117" t="s">
         <v>420</v>
       </c>
@@ -4880,7 +4885,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="118" spans="1:7">
+    <row r="118" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A118" t="s">
         <v>420</v>
       </c>
@@ -4897,7 +4902,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="119" spans="1:7">
+    <row r="119" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A119" t="s">
         <v>420</v>
       </c>
@@ -4914,7 +4919,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="120" spans="1:7">
+    <row r="120" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A120" t="s">
         <v>420</v>
       </c>
@@ -4931,7 +4936,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="121" spans="1:7">
+    <row r="121" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A121" t="s">
         <v>420</v>
       </c>
@@ -4948,7 +4953,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="122" spans="1:7">
+    <row r="122" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A122" t="s">
         <v>420</v>
       </c>
@@ -4965,7 +4970,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="123" spans="1:7">
+    <row r="123" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A123" t="s">
         <v>16</v>
       </c>
@@ -4982,7 +4987,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="124" spans="1:7">
+    <row r="124" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A124" t="s">
         <v>156</v>
       </c>
@@ -4999,7 +5004,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="125" spans="1:7">
+    <row r="125" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A125" t="s">
         <v>445</v>
       </c>
@@ -5016,7 +5021,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="126" spans="1:7">
+    <row r="126" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A126" t="s">
         <v>449</v>
       </c>
@@ -5033,7 +5038,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="127" spans="1:7">
+    <row r="127" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A127" t="s">
         <v>16</v>
       </c>
@@ -5050,7 +5055,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="128" spans="1:7">
+    <row r="128" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A128" t="s">
         <v>156</v>
       </c>
@@ -5067,7 +5072,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="129" spans="1:8">
+    <row r="129" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A129" t="s">
         <v>156</v>
       </c>
@@ -5084,7 +5089,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="130" spans="1:8">
+    <row r="130" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A130" t="s">
         <v>156</v>
       </c>
@@ -5101,7 +5106,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="131" spans="1:8">
+    <row r="131" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A131" t="s">
         <v>156</v>
       </c>
@@ -5118,7 +5123,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="132" spans="1:8">
+    <row r="132" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A132" t="s">
         <v>156</v>
       </c>
@@ -5135,7 +5140,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="133" spans="1:8">
+    <row r="133" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A133" t="s">
         <v>156</v>
       </c>
@@ -5152,7 +5157,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="134" spans="1:8">
+    <row r="134" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A134" t="s">
         <v>156</v>
       </c>
@@ -5169,7 +5174,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="135" spans="1:8">
+    <row r="135" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A135" t="s">
         <v>16</v>
       </c>
@@ -5186,7 +5191,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="136" spans="1:8">
+    <row r="136" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A136" t="s">
         <v>156</v>
       </c>
@@ -5203,7 +5208,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="137" spans="1:8">
+    <row r="137" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A137" t="s">
         <v>156</v>
       </c>
@@ -5220,7 +5225,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="138" spans="1:8">
+    <row r="138" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A138" t="s">
         <v>156</v>
       </c>
@@ -5237,7 +5242,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="139" spans="1:8">
+    <row r="139" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A139" t="s">
         <v>156</v>
       </c>
@@ -5254,7 +5259,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="140" spans="1:8">
+    <row r="140" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A140" t="s">
         <v>16</v>
       </c>
@@ -5271,7 +5276,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="141" spans="1:8">
+    <row r="141" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A141" t="s">
         <v>495</v>
       </c>
@@ -5291,7 +5296,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="142" spans="1:8">
+    <row r="142" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A142" t="s">
         <v>25</v>
       </c>
@@ -5304,9 +5309,9 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:E198"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
-    <row r="1" spans="1:5">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>499</v>
       </c>
@@ -5323,7 +5328,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="2" spans="1:5">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>501</v>
       </c>
@@ -5337,7 +5342,7 @@
         <v>504</v>
       </c>
     </row>
-    <row r="3" spans="1:5">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>501</v>
       </c>
@@ -5351,7 +5356,7 @@
         <v>507</v>
       </c>
     </row>
-    <row r="4" spans="1:5">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>27</v>
       </c>
@@ -5365,7 +5370,7 @@
         <v>508</v>
       </c>
     </row>
-    <row r="5" spans="1:5">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>27</v>
       </c>
@@ -5379,7 +5384,7 @@
         <v>509</v>
       </c>
     </row>
-    <row r="6" spans="1:5">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>510</v>
       </c>
@@ -5393,7 +5398,7 @@
         <v>512</v>
       </c>
     </row>
-    <row r="7" spans="1:5">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>510</v>
       </c>
@@ -5407,7 +5412,7 @@
         <v>514</v>
       </c>
     </row>
-    <row r="8" spans="1:5">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>510</v>
       </c>
@@ -5421,7 +5426,7 @@
         <v>516</v>
       </c>
     </row>
-    <row r="9" spans="1:5">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>510</v>
       </c>
@@ -5435,7 +5440,7 @@
         <v>518</v>
       </c>
     </row>
-    <row r="10" spans="1:5">
+    <row r="10" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>510</v>
       </c>
@@ -5449,7 +5454,7 @@
         <v>520</v>
       </c>
     </row>
-    <row r="11" spans="1:5">
+    <row r="11" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>510</v>
       </c>
@@ -5463,7 +5468,7 @@
         <v>522</v>
       </c>
     </row>
-    <row r="12" spans="1:5">
+    <row r="12" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>510</v>
       </c>
@@ -5477,7 +5482,7 @@
         <v>524</v>
       </c>
     </row>
-    <row r="13" spans="1:5">
+    <row r="13" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>510</v>
       </c>
@@ -5491,7 +5496,7 @@
         <v>526</v>
       </c>
     </row>
-    <row r="14" spans="1:5">
+    <row r="14" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
         <v>510</v>
       </c>
@@ -5505,7 +5510,7 @@
         <v>528</v>
       </c>
     </row>
-    <row r="15" spans="1:5">
+    <row r="15" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
         <v>510</v>
       </c>
@@ -5519,7 +5524,7 @@
         <v>530</v>
       </c>
     </row>
-    <row r="16" spans="1:5">
+    <row r="16" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
         <v>510</v>
       </c>
@@ -5533,7 +5538,7 @@
         <v>532</v>
       </c>
     </row>
-    <row r="17" spans="1:4">
+    <row r="17" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
         <v>510</v>
       </c>
@@ -5547,7 +5552,7 @@
         <v>534</v>
       </c>
     </row>
-    <row r="18" spans="1:4">
+    <row r="18" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
         <v>510</v>
       </c>
@@ -5561,7 +5566,7 @@
         <v>536</v>
       </c>
     </row>
-    <row r="19" spans="1:4">
+    <row r="19" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
         <v>537</v>
       </c>
@@ -5575,7 +5580,7 @@
         <v>540</v>
       </c>
     </row>
-    <row r="20" spans="1:4">
+    <row r="20" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
         <v>537</v>
       </c>
@@ -5589,7 +5594,7 @@
         <v>543</v>
       </c>
     </row>
-    <row r="21" spans="1:4">
+    <row r="21" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
         <v>537</v>
       </c>
@@ -5603,7 +5608,7 @@
         <v>546</v>
       </c>
     </row>
-    <row r="22" spans="1:4">
+    <row r="22" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
         <v>537</v>
       </c>
@@ -5617,7 +5622,7 @@
         <v>549</v>
       </c>
     </row>
-    <row r="23" spans="1:4">
+    <row r="23" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
         <v>537</v>
       </c>
@@ -5631,7 +5636,7 @@
         <v>552</v>
       </c>
     </row>
-    <row r="24" spans="1:4">
+    <row r="24" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
         <v>537</v>
       </c>
@@ -5645,7 +5650,7 @@
         <v>555</v>
       </c>
     </row>
-    <row r="25" spans="1:4">
+    <row r="25" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
         <v>537</v>
       </c>
@@ -5659,7 +5664,7 @@
         <v>558</v>
       </c>
     </row>
-    <row r="26" spans="1:4">
+    <row r="26" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A26" t="s">
         <v>74</v>
       </c>
@@ -5673,7 +5678,7 @@
         <v>560</v>
       </c>
     </row>
-    <row r="27" spans="1:4">
+    <row r="27" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A27" t="s">
         <v>74</v>
       </c>
@@ -5687,7 +5692,7 @@
         <v>562</v>
       </c>
     </row>
-    <row r="28" spans="1:4">
+    <row r="28" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A28" t="s">
         <v>74</v>
       </c>
@@ -5701,7 +5706,7 @@
         <v>565</v>
       </c>
     </row>
-    <row r="29" spans="1:4">
+    <row r="29" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A29" t="s">
         <v>74</v>
       </c>
@@ -5715,7 +5720,7 @@
         <v>568</v>
       </c>
     </row>
-    <row r="30" spans="1:4">
+    <row r="30" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A30" t="s">
         <v>82</v>
       </c>
@@ -5729,7 +5734,7 @@
         <v>570</v>
       </c>
     </row>
-    <row r="31" spans="1:4">
+    <row r="31" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A31" t="s">
         <v>82</v>
       </c>
@@ -5743,7 +5748,7 @@
         <v>572</v>
       </c>
     </row>
-    <row r="32" spans="1:4">
+    <row r="32" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A32" t="s">
         <v>82</v>
       </c>
@@ -5757,7 +5762,7 @@
         <v>574</v>
       </c>
     </row>
-    <row r="33" spans="1:4">
+    <row r="33" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A33" t="s">
         <v>82</v>
       </c>
@@ -5771,7 +5776,7 @@
         <v>577</v>
       </c>
     </row>
-    <row r="34" spans="1:4">
+    <row r="34" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A34" t="s">
         <v>82</v>
       </c>
@@ -5785,7 +5790,7 @@
         <v>580</v>
       </c>
     </row>
-    <row r="35" spans="1:4">
+    <row r="35" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A35" t="s">
         <v>82</v>
       </c>
@@ -5799,7 +5804,7 @@
         <v>583</v>
       </c>
     </row>
-    <row r="36" spans="1:4">
+    <row r="36" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A36" t="s">
         <v>82</v>
       </c>
@@ -5813,7 +5818,7 @@
         <v>586</v>
       </c>
     </row>
-    <row r="37" spans="1:4">
+    <row r="37" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A37" t="s">
         <v>82</v>
       </c>
@@ -5827,7 +5832,7 @@
         <v>588</v>
       </c>
     </row>
-    <row r="38" spans="1:4">
+    <row r="38" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A38" t="s">
         <v>82</v>
       </c>
@@ -5841,7 +5846,7 @@
         <v>568</v>
       </c>
     </row>
-    <row r="39" spans="1:4">
+    <row r="39" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A39" t="s">
         <v>589</v>
       </c>
@@ -5855,7 +5860,7 @@
         <v>591</v>
       </c>
     </row>
-    <row r="40" spans="1:4">
+    <row r="40" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A40" t="s">
         <v>589</v>
       </c>
@@ -5869,7 +5874,7 @@
         <v>593</v>
       </c>
     </row>
-    <row r="41" spans="1:4">
+    <row r="41" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A41" t="s">
         <v>589</v>
       </c>
@@ -5883,7 +5888,7 @@
         <v>568</v>
       </c>
     </row>
-    <row r="42" spans="1:4">
+    <row r="42" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A42" t="s">
         <v>594</v>
       </c>
@@ -5897,7 +5902,7 @@
         <v>596</v>
       </c>
     </row>
-    <row r="43" spans="1:4">
+    <row r="43" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A43" t="s">
         <v>594</v>
       </c>
@@ -5911,7 +5916,7 @@
         <v>598</v>
       </c>
     </row>
-    <row r="44" spans="1:4">
+    <row r="44" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A44" t="s">
         <v>594</v>
       </c>
@@ -5925,7 +5930,7 @@
         <v>600</v>
       </c>
     </row>
-    <row r="45" spans="1:4">
+    <row r="45" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A45" t="s">
         <v>594</v>
       </c>
@@ -5939,7 +5944,7 @@
         <v>602</v>
       </c>
     </row>
-    <row r="46" spans="1:4">
+    <row r="46" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A46" t="s">
         <v>594</v>
       </c>
@@ -5953,7 +5958,7 @@
         <v>604</v>
       </c>
     </row>
-    <row r="47" spans="1:4">
+    <row r="47" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A47" t="s">
         <v>594</v>
       </c>
@@ -5967,7 +5972,7 @@
         <v>606</v>
       </c>
     </row>
-    <row r="48" spans="1:4">
+    <row r="48" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A48" t="s">
         <v>607</v>
       </c>
@@ -5981,7 +5986,7 @@
         <v>608</v>
       </c>
     </row>
-    <row r="49" spans="1:5">
+    <row r="49" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A49" t="s">
         <v>607</v>
       </c>
@@ -5995,7 +6000,7 @@
         <v>609</v>
       </c>
     </row>
-    <row r="50" spans="1:5">
+    <row r="50" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A50" t="s">
         <v>607</v>
       </c>
@@ -6009,7 +6014,7 @@
         <v>611</v>
       </c>
     </row>
-    <row r="51" spans="1:5">
+    <row r="51" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A51" t="s">
         <v>607</v>
       </c>
@@ -6023,7 +6028,7 @@
         <v>568</v>
       </c>
     </row>
-    <row r="52" spans="1:5">
+    <row r="52" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A52" t="s">
         <v>613</v>
       </c>
@@ -6037,7 +6042,7 @@
         <v>615</v>
       </c>
     </row>
-    <row r="53" spans="1:5">
+    <row r="53" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A53" t="s">
         <v>613</v>
       </c>
@@ -6054,7 +6059,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="54" spans="1:5">
+    <row r="54" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A54" t="s">
         <v>613</v>
       </c>
@@ -6071,7 +6076,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="55" spans="1:5">
+    <row r="55" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A55" t="s">
         <v>613</v>
       </c>
@@ -6088,7 +6093,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="56" spans="1:5">
+    <row r="56" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A56" t="s">
         <v>613</v>
       </c>
@@ -6105,7 +6110,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="57" spans="1:5">
+    <row r="57" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A57" t="s">
         <v>613</v>
       </c>
@@ -6122,7 +6127,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="58" spans="1:5">
+    <row r="58" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A58" t="s">
         <v>623</v>
       </c>
@@ -6136,7 +6141,7 @@
         <v>625</v>
       </c>
     </row>
-    <row r="59" spans="1:5">
+    <row r="59" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A59" t="s">
         <v>623</v>
       </c>
@@ -6150,7 +6155,7 @@
         <v>627</v>
       </c>
     </row>
-    <row r="60" spans="1:5">
+    <row r="60" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A60" t="s">
         <v>623</v>
       </c>
@@ -6164,7 +6169,7 @@
         <v>629</v>
       </c>
     </row>
-    <row r="61" spans="1:5">
+    <row r="61" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A61" t="s">
         <v>630</v>
       </c>
@@ -6178,7 +6183,7 @@
         <v>632</v>
       </c>
     </row>
-    <row r="62" spans="1:5">
+    <row r="62" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A62" t="s">
         <v>630</v>
       </c>
@@ -6192,7 +6197,7 @@
         <v>634</v>
       </c>
     </row>
-    <row r="63" spans="1:5">
+    <row r="63" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A63" t="s">
         <v>630</v>
       </c>
@@ -6206,7 +6211,7 @@
         <v>568</v>
       </c>
     </row>
-    <row r="64" spans="1:5">
+    <row r="64" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A64" t="s">
         <v>635</v>
       </c>
@@ -6220,7 +6225,7 @@
         <v>508</v>
       </c>
     </row>
-    <row r="65" spans="1:4">
+    <row r="65" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A65" t="s">
         <v>635</v>
       </c>
@@ -6234,7 +6239,7 @@
         <v>509</v>
       </c>
     </row>
-    <row r="66" spans="1:4">
+    <row r="66" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A66" t="s">
         <v>635</v>
       </c>
@@ -6248,7 +6253,7 @@
         <v>568</v>
       </c>
     </row>
-    <row r="67" spans="1:4">
+    <row r="67" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A67" t="s">
         <v>636</v>
       </c>
@@ -6262,7 +6267,7 @@
         <v>508</v>
       </c>
     </row>
-    <row r="68" spans="1:4">
+    <row r="68" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A68" t="s">
         <v>636</v>
       </c>
@@ -6276,7 +6281,7 @@
         <v>509</v>
       </c>
     </row>
-    <row r="69" spans="1:4">
+    <row r="69" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A69" t="s">
         <v>636</v>
       </c>
@@ -6290,7 +6295,7 @@
         <v>638</v>
       </c>
     </row>
-    <row r="70" spans="1:4">
+    <row r="70" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A70" t="s">
         <v>636</v>
       </c>
@@ -6304,7 +6309,7 @@
         <v>568</v>
       </c>
     </row>
-    <row r="71" spans="1:4">
+    <row r="71" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A71" t="s">
         <v>133</v>
       </c>
@@ -6318,7 +6323,7 @@
         <v>640</v>
       </c>
     </row>
-    <row r="72" spans="1:4">
+    <row r="72" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A72" t="s">
         <v>133</v>
       </c>
@@ -6332,7 +6337,7 @@
         <v>642</v>
       </c>
     </row>
-    <row r="73" spans="1:4">
+    <row r="73" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A73" t="s">
         <v>133</v>
       </c>
@@ -6346,7 +6351,7 @@
         <v>638</v>
       </c>
     </row>
-    <row r="74" spans="1:4">
+    <row r="74" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A74" t="s">
         <v>133</v>
       </c>
@@ -6360,7 +6365,7 @@
         <v>568</v>
       </c>
     </row>
-    <row r="75" spans="1:4">
+    <row r="75" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A75" t="s">
         <v>137</v>
       </c>
@@ -6374,7 +6379,7 @@
         <v>644</v>
       </c>
     </row>
-    <row r="76" spans="1:4">
+    <row r="76" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A76" t="s">
         <v>137</v>
       </c>
@@ -6388,7 +6393,7 @@
         <v>646</v>
       </c>
     </row>
-    <row r="77" spans="1:4">
+    <row r="77" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A77" t="s">
         <v>137</v>
       </c>
@@ -6402,7 +6407,7 @@
         <v>648</v>
       </c>
     </row>
-    <row r="78" spans="1:4">
+    <row r="78" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A78" t="s">
         <v>137</v>
       </c>
@@ -6416,7 +6421,7 @@
         <v>650</v>
       </c>
     </row>
-    <row r="79" spans="1:4">
+    <row r="79" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A79" t="s">
         <v>144</v>
       </c>
@@ -6430,7 +6435,7 @@
         <v>652</v>
       </c>
     </row>
-    <row r="80" spans="1:4">
+    <row r="80" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A80" t="s">
         <v>144</v>
       </c>
@@ -6444,7 +6449,7 @@
         <v>654</v>
       </c>
     </row>
-    <row r="81" spans="1:4">
+    <row r="81" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A81" t="s">
         <v>144</v>
       </c>
@@ -6458,7 +6463,7 @@
         <v>656</v>
       </c>
     </row>
-    <row r="82" spans="1:4">
+    <row r="82" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A82" t="s">
         <v>144</v>
       </c>
@@ -6472,7 +6477,7 @@
         <v>648</v>
       </c>
     </row>
-    <row r="83" spans="1:4">
+    <row r="83" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A83" t="s">
         <v>144</v>
       </c>
@@ -6486,7 +6491,7 @@
         <v>659</v>
       </c>
     </row>
-    <row r="84" spans="1:4">
+    <row r="84" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A84" t="s">
         <v>144</v>
       </c>
@@ -6500,7 +6505,7 @@
         <v>661</v>
       </c>
     </row>
-    <row r="85" spans="1:4">
+    <row r="85" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A85" t="s">
         <v>662</v>
       </c>
@@ -6514,7 +6519,7 @@
         <v>664</v>
       </c>
     </row>
-    <row r="86" spans="1:4">
+    <row r="86" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A86" t="s">
         <v>662</v>
       </c>
@@ -6528,7 +6533,7 @@
         <v>666</v>
       </c>
     </row>
-    <row r="87" spans="1:4">
+    <row r="87" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A87" t="s">
         <v>662</v>
       </c>
@@ -6542,7 +6547,7 @@
         <v>668</v>
       </c>
     </row>
-    <row r="88" spans="1:4">
+    <row r="88" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A88" t="s">
         <v>662</v>
       </c>
@@ -6556,7 +6561,7 @@
         <v>670</v>
       </c>
     </row>
-    <row r="89" spans="1:4">
+    <row r="89" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A89" t="s">
         <v>662</v>
       </c>
@@ -6570,7 +6575,7 @@
         <v>672</v>
       </c>
     </row>
-    <row r="90" spans="1:4">
+    <row r="90" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A90" t="s">
         <v>662</v>
       </c>
@@ -6584,7 +6589,7 @@
         <v>568</v>
       </c>
     </row>
-    <row r="91" spans="1:4">
+    <row r="91" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A91" t="s">
         <v>662</v>
       </c>
@@ -6598,7 +6603,7 @@
         <v>674</v>
       </c>
     </row>
-    <row r="92" spans="1:4">
+    <row r="92" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A92" t="s">
         <v>675</v>
       </c>
@@ -6612,7 +6617,7 @@
         <v>677</v>
       </c>
     </row>
-    <row r="93" spans="1:4">
+    <row r="93" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A93" t="s">
         <v>675</v>
       </c>
@@ -6626,7 +6631,7 @@
         <v>679</v>
       </c>
     </row>
-    <row r="94" spans="1:4">
+    <row r="94" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A94" t="s">
         <v>675</v>
       </c>
@@ -6640,7 +6645,7 @@
         <v>681</v>
       </c>
     </row>
-    <row r="95" spans="1:4">
+    <row r="95" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A95" t="s">
         <v>675</v>
       </c>
@@ -6654,7 +6659,7 @@
         <v>683</v>
       </c>
     </row>
-    <row r="96" spans="1:4">
+    <row r="96" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A96" t="s">
         <v>675</v>
       </c>
@@ -6668,7 +6673,7 @@
         <v>685</v>
       </c>
     </row>
-    <row r="97" spans="1:5">
+    <row r="97" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A97" t="s">
         <v>686</v>
       </c>
@@ -6682,7 +6687,7 @@
         <v>508</v>
       </c>
     </row>
-    <row r="98" spans="1:5">
+    <row r="98" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A98" t="s">
         <v>686</v>
       </c>
@@ -6696,7 +6701,7 @@
         <v>509</v>
       </c>
     </row>
-    <row r="99" spans="1:5">
+    <row r="99" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A99" t="s">
         <v>686</v>
       </c>
@@ -6710,7 +6715,7 @@
         <v>687</v>
       </c>
     </row>
-    <row r="100" spans="1:5">
+    <row r="100" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A100" t="s">
         <v>686</v>
       </c>
@@ -6724,7 +6729,7 @@
         <v>568</v>
       </c>
     </row>
-    <row r="101" spans="1:5">
+    <row r="101" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A101" t="s">
         <v>688</v>
       </c>
@@ -6738,7 +6743,7 @@
         <v>690</v>
       </c>
     </row>
-    <row r="102" spans="1:5">
+    <row r="102" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A102" t="s">
         <v>688</v>
       </c>
@@ -6755,7 +6760,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="103" spans="1:5">
+    <row r="103" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A103" t="s">
         <v>688</v>
       </c>
@@ -6772,7 +6777,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="104" spans="1:5">
+    <row r="104" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A104" t="s">
         <v>688</v>
       </c>
@@ -6789,7 +6794,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="105" spans="1:5">
+    <row r="105" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A105" t="s">
         <v>688</v>
       </c>
@@ -6806,7 +6811,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="106" spans="1:5">
+    <row r="106" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A106" t="s">
         <v>688</v>
       </c>
@@ -6823,7 +6828,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="107" spans="1:5">
+    <row r="107" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A107" t="s">
         <v>688</v>
       </c>
@@ -6840,7 +6845,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="108" spans="1:5">
+    <row r="108" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A108" t="s">
         <v>688</v>
       </c>
@@ -6857,7 +6862,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="109" spans="1:5">
+    <row r="109" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A109" t="s">
         <v>688</v>
       </c>
@@ -6874,7 +6879,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="110" spans="1:5">
+    <row r="110" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A110" t="s">
         <v>705</v>
       </c>
@@ -6888,7 +6893,7 @@
         <v>707</v>
       </c>
     </row>
-    <row r="111" spans="1:5">
+    <row r="111" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A111" t="s">
         <v>705</v>
       </c>
@@ -6902,7 +6907,7 @@
         <v>709</v>
       </c>
     </row>
-    <row r="112" spans="1:5">
+    <row r="112" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A112" t="s">
         <v>705</v>
       </c>
@@ -6916,7 +6921,7 @@
         <v>711</v>
       </c>
     </row>
-    <row r="113" spans="1:4">
+    <row r="113" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A113" t="s">
         <v>705</v>
       </c>
@@ -6930,7 +6935,7 @@
         <v>713</v>
       </c>
     </row>
-    <row r="114" spans="1:4">
+    <row r="114" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A114" t="s">
         <v>705</v>
       </c>
@@ -6944,7 +6949,7 @@
         <v>715</v>
       </c>
     </row>
-    <row r="115" spans="1:4">
+    <row r="115" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A115" t="s">
         <v>705</v>
       </c>
@@ -6958,7 +6963,7 @@
         <v>568</v>
       </c>
     </row>
-    <row r="116" spans="1:4">
+    <row r="116" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A116" t="s">
         <v>716</v>
       </c>
@@ -6972,7 +6977,7 @@
         <v>717</v>
       </c>
     </row>
-    <row r="117" spans="1:4">
+    <row r="117" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A117" t="s">
         <v>716</v>
       </c>
@@ -6986,7 +6991,7 @@
         <v>692</v>
       </c>
     </row>
-    <row r="118" spans="1:4">
+    <row r="118" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A118" t="s">
         <v>716</v>
       </c>
@@ -7000,7 +7005,7 @@
         <v>696</v>
       </c>
     </row>
-    <row r="119" spans="1:4">
+    <row r="119" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A119" t="s">
         <v>716</v>
       </c>
@@ -7014,7 +7019,7 @@
         <v>719</v>
       </c>
     </row>
-    <row r="120" spans="1:4">
+    <row r="120" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A120" t="s">
         <v>716</v>
       </c>
@@ -7028,7 +7033,7 @@
         <v>721</v>
       </c>
     </row>
-    <row r="121" spans="1:4">
+    <row r="121" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A121" t="s">
         <v>716</v>
       </c>
@@ -7042,7 +7047,7 @@
         <v>722</v>
       </c>
     </row>
-    <row r="122" spans="1:4">
+    <row r="122" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A122" t="s">
         <v>716</v>
       </c>
@@ -7056,7 +7061,7 @@
         <v>568</v>
       </c>
     </row>
-    <row r="123" spans="1:4">
+    <row r="123" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A123" t="s">
         <v>723</v>
       </c>
@@ -7070,7 +7075,7 @@
         <v>724</v>
       </c>
     </row>
-    <row r="124" spans="1:4">
+    <row r="124" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A124" t="s">
         <v>723</v>
       </c>
@@ -7084,7 +7089,7 @@
         <v>725</v>
       </c>
     </row>
-    <row r="125" spans="1:4">
+    <row r="125" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A125" t="s">
         <v>726</v>
       </c>
@@ -7098,7 +7103,7 @@
         <v>728</v>
       </c>
     </row>
-    <row r="126" spans="1:4">
+    <row r="126" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A126" t="s">
         <v>726</v>
       </c>
@@ -7112,7 +7117,7 @@
         <v>730</v>
       </c>
     </row>
-    <row r="127" spans="1:4">
+    <row r="127" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A127" t="s">
         <v>726</v>
       </c>
@@ -7126,7 +7131,7 @@
         <v>668</v>
       </c>
     </row>
-    <row r="128" spans="1:4">
+    <row r="128" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A128" t="s">
         <v>726</v>
       </c>
@@ -7140,7 +7145,7 @@
         <v>732</v>
       </c>
     </row>
-    <row r="129" spans="1:4">
+    <row r="129" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A129" t="s">
         <v>726</v>
       </c>
@@ -7154,7 +7159,7 @@
         <v>734</v>
       </c>
     </row>
-    <row r="130" spans="1:4">
+    <row r="130" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A130" t="s">
         <v>735</v>
       </c>
@@ -7168,7 +7173,7 @@
         <v>664</v>
       </c>
     </row>
-    <row r="131" spans="1:4">
+    <row r="131" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A131" t="s">
         <v>735</v>
       </c>
@@ -7182,7 +7187,7 @@
         <v>666</v>
       </c>
     </row>
-    <row r="132" spans="1:4">
+    <row r="132" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A132" t="s">
         <v>735</v>
       </c>
@@ -7196,7 +7201,7 @@
         <v>668</v>
       </c>
     </row>
-    <row r="133" spans="1:4">
+    <row r="133" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A133" t="s">
         <v>735</v>
       </c>
@@ -7210,7 +7215,7 @@
         <v>670</v>
       </c>
     </row>
-    <row r="134" spans="1:4">
+    <row r="134" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A134" t="s">
         <v>735</v>
       </c>
@@ -7224,7 +7229,7 @@
         <v>672</v>
       </c>
     </row>
-    <row r="135" spans="1:4">
+    <row r="135" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A135" t="s">
         <v>735</v>
       </c>
@@ -7238,7 +7243,7 @@
         <v>568</v>
       </c>
     </row>
-    <row r="136" spans="1:4">
+    <row r="136" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A136" t="s">
         <v>736</v>
       </c>
@@ -7252,7 +7257,7 @@
         <v>664</v>
       </c>
     </row>
-    <row r="137" spans="1:4">
+    <row r="137" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A137" t="s">
         <v>736</v>
       </c>
@@ -7266,7 +7271,7 @@
         <v>666</v>
       </c>
     </row>
-    <row r="138" spans="1:4">
+    <row r="138" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A138" t="s">
         <v>736</v>
       </c>
@@ -7280,7 +7285,7 @@
         <v>668</v>
       </c>
     </row>
-    <row r="139" spans="1:4">
+    <row r="139" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A139" t="s">
         <v>736</v>
       </c>
@@ -7294,7 +7299,7 @@
         <v>670</v>
       </c>
     </row>
-    <row r="140" spans="1:4">
+    <row r="140" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A140" t="s">
         <v>736</v>
       </c>
@@ -7308,7 +7313,7 @@
         <v>672</v>
       </c>
     </row>
-    <row r="141" spans="1:4">
+    <row r="141" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A141" t="s">
         <v>736</v>
       </c>
@@ -7322,7 +7327,7 @@
         <v>568</v>
       </c>
     </row>
-    <row r="142" spans="1:4">
+    <row r="142" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A142" t="s">
         <v>737</v>
       </c>
@@ -7336,7 +7341,7 @@
         <v>739</v>
       </c>
     </row>
-    <row r="143" spans="1:4">
+    <row r="143" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A143" t="s">
         <v>737</v>
       </c>
@@ -7350,7 +7355,7 @@
         <v>741</v>
       </c>
     </row>
-    <row r="144" spans="1:4">
+    <row r="144" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A144" t="s">
         <v>737</v>
       </c>
@@ -7364,7 +7369,7 @@
         <v>742</v>
       </c>
     </row>
-    <row r="145" spans="1:4">
+    <row r="145" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A145" t="s">
         <v>737</v>
       </c>
@@ -7378,7 +7383,7 @@
         <v>744</v>
       </c>
     </row>
-    <row r="146" spans="1:4">
+    <row r="146" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A146" t="s">
         <v>737</v>
       </c>
@@ -7392,7 +7397,7 @@
         <v>746</v>
       </c>
     </row>
-    <row r="147" spans="1:4">
+    <row r="147" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A147" t="s">
         <v>737</v>
       </c>
@@ -7406,7 +7411,7 @@
         <v>568</v>
       </c>
     </row>
-    <row r="148" spans="1:4">
+    <row r="148" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A148" t="s">
         <v>737</v>
       </c>
@@ -7420,7 +7425,7 @@
         <v>674</v>
       </c>
     </row>
-    <row r="149" spans="1:4">
+    <row r="149" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A149" t="s">
         <v>747</v>
       </c>
@@ -7434,7 +7439,7 @@
         <v>749</v>
       </c>
     </row>
-    <row r="150" spans="1:4">
+    <row r="150" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A150" t="s">
         <v>747</v>
       </c>
@@ -7448,7 +7453,7 @@
         <v>751</v>
       </c>
     </row>
-    <row r="151" spans="1:4">
+    <row r="151" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A151" t="s">
         <v>747</v>
       </c>
@@ -7462,7 +7467,7 @@
         <v>753</v>
       </c>
     </row>
-    <row r="152" spans="1:4">
+    <row r="152" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A152" t="s">
         <v>747</v>
       </c>
@@ -7476,7 +7481,7 @@
         <v>755</v>
       </c>
     </row>
-    <row r="153" spans="1:4">
+    <row r="153" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A153" t="s">
         <v>747</v>
       </c>
@@ -7490,7 +7495,7 @@
         <v>757</v>
       </c>
     </row>
-    <row r="154" spans="1:4">
+    <row r="154" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A154" t="s">
         <v>747</v>
       </c>
@@ -7504,7 +7509,7 @@
         <v>568</v>
       </c>
     </row>
-    <row r="155" spans="1:4">
+    <row r="155" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A155" t="s">
         <v>747</v>
       </c>
@@ -7518,7 +7523,7 @@
         <v>638</v>
       </c>
     </row>
-    <row r="156" spans="1:4">
+    <row r="156" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A156" t="s">
         <v>759</v>
       </c>
@@ -7532,7 +7537,7 @@
         <v>707</v>
       </c>
     </row>
-    <row r="157" spans="1:4">
+    <row r="157" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A157" t="s">
         <v>759</v>
       </c>
@@ -7546,7 +7551,7 @@
         <v>709</v>
       </c>
     </row>
-    <row r="158" spans="1:4">
+    <row r="158" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A158" t="s">
         <v>759</v>
       </c>
@@ -7560,7 +7565,7 @@
         <v>761</v>
       </c>
     </row>
-    <row r="159" spans="1:4">
+    <row r="159" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A159" t="s">
         <v>759</v>
       </c>
@@ -7574,7 +7579,7 @@
         <v>711</v>
       </c>
     </row>
-    <row r="160" spans="1:4">
+    <row r="160" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A160" t="s">
         <v>759</v>
       </c>
@@ -7588,7 +7593,7 @@
         <v>713</v>
       </c>
     </row>
-    <row r="161" spans="1:4">
+    <row r="161" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A161" t="s">
         <v>759</v>
       </c>
@@ -7602,7 +7607,7 @@
         <v>568</v>
       </c>
     </row>
-    <row r="162" spans="1:4">
+    <row r="162" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A162" t="s">
         <v>762</v>
       </c>
@@ -7616,7 +7621,7 @@
         <v>664</v>
       </c>
     </row>
-    <row r="163" spans="1:4">
+    <row r="163" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A163" t="s">
         <v>762</v>
       </c>
@@ -7630,7 +7635,7 @@
         <v>666</v>
       </c>
     </row>
-    <row r="164" spans="1:4">
+    <row r="164" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A164" t="s">
         <v>762</v>
       </c>
@@ -7644,7 +7649,7 @@
         <v>668</v>
       </c>
     </row>
-    <row r="165" spans="1:4">
+    <row r="165" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A165" t="s">
         <v>762</v>
       </c>
@@ -7658,7 +7663,7 @@
         <v>670</v>
       </c>
     </row>
-    <row r="166" spans="1:4">
+    <row r="166" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A166" t="s">
         <v>762</v>
       </c>
@@ -7672,7 +7677,7 @@
         <v>672</v>
       </c>
     </row>
-    <row r="167" spans="1:4">
+    <row r="167" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A167" t="s">
         <v>762</v>
       </c>
@@ -7686,7 +7691,7 @@
         <v>568</v>
       </c>
     </row>
-    <row r="168" spans="1:4">
+    <row r="168" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A168" t="s">
         <v>762</v>
       </c>
@@ -7700,7 +7705,7 @@
         <v>674</v>
       </c>
     </row>
-    <row r="169" spans="1:4">
+    <row r="169" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A169" t="s">
         <v>764</v>
       </c>
@@ -7714,7 +7719,7 @@
         <v>766</v>
       </c>
     </row>
-    <row r="170" spans="1:4">
+    <row r="170" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A170" t="s">
         <v>764</v>
       </c>
@@ -7728,7 +7733,7 @@
         <v>768</v>
       </c>
     </row>
-    <row r="171" spans="1:4">
+    <row r="171" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A171" t="s">
         <v>764</v>
       </c>
@@ -7742,7 +7747,7 @@
         <v>770</v>
       </c>
     </row>
-    <row r="172" spans="1:4">
+    <row r="172" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A172" t="s">
         <v>764</v>
       </c>
@@ -7756,7 +7761,7 @@
         <v>772</v>
       </c>
     </row>
-    <row r="173" spans="1:4">
+    <row r="173" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A173" t="s">
         <v>764</v>
       </c>
@@ -7770,7 +7775,7 @@
         <v>774</v>
       </c>
     </row>
-    <row r="174" spans="1:4">
+    <row r="174" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A174" t="s">
         <v>764</v>
       </c>
@@ -7784,7 +7789,7 @@
         <v>568</v>
       </c>
     </row>
-    <row r="175" spans="1:4">
+    <row r="175" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A175" t="s">
         <v>775</v>
       </c>
@@ -7798,7 +7803,7 @@
         <v>777</v>
       </c>
     </row>
-    <row r="176" spans="1:4">
+    <row r="176" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A176" t="s">
         <v>775</v>
       </c>
@@ -7812,7 +7817,7 @@
         <v>779</v>
       </c>
     </row>
-    <row r="177" spans="1:4">
+    <row r="177" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A177" t="s">
         <v>775</v>
       </c>
@@ -7826,7 +7831,7 @@
         <v>781</v>
       </c>
     </row>
-    <row r="178" spans="1:4">
+    <row r="178" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A178" t="s">
         <v>775</v>
       </c>
@@ -7840,7 +7845,7 @@
         <v>782</v>
       </c>
     </row>
-    <row r="179" spans="1:4">
+    <row r="179" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A179" t="s">
         <v>775</v>
       </c>
@@ -7854,7 +7859,7 @@
         <v>568</v>
       </c>
     </row>
-    <row r="180" spans="1:4">
+    <row r="180" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A180" t="s">
         <v>783</v>
       </c>
@@ -7868,7 +7873,7 @@
         <v>664</v>
       </c>
     </row>
-    <row r="181" spans="1:4">
+    <row r="181" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A181" t="s">
         <v>783</v>
       </c>
@@ -7882,7 +7887,7 @@
         <v>666</v>
       </c>
     </row>
-    <row r="182" spans="1:4">
+    <row r="182" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A182" t="s">
         <v>783</v>
       </c>
@@ -7896,7 +7901,7 @@
         <v>742</v>
       </c>
     </row>
-    <row r="183" spans="1:4">
+    <row r="183" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A183" t="s">
         <v>783</v>
       </c>
@@ -7910,7 +7915,7 @@
         <v>670</v>
       </c>
     </row>
-    <row r="184" spans="1:4">
+    <row r="184" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A184" t="s">
         <v>783</v>
       </c>
@@ -7924,7 +7929,7 @@
         <v>672</v>
       </c>
     </row>
-    <row r="185" spans="1:4">
+    <row r="185" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A185" t="s">
         <v>783</v>
       </c>
@@ -7938,7 +7943,7 @@
         <v>568</v>
       </c>
     </row>
-    <row r="186" spans="1:4">
+    <row r="186" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A186" t="s">
         <v>783</v>
       </c>
@@ -7952,7 +7957,7 @@
         <v>638</v>
       </c>
     </row>
-    <row r="187" spans="1:4">
+    <row r="187" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A187" t="s">
         <v>785</v>
       </c>
@@ -7966,7 +7971,7 @@
         <v>739</v>
       </c>
     </row>
-    <row r="188" spans="1:4">
+    <row r="188" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A188" t="s">
         <v>785</v>
       </c>
@@ -7980,7 +7985,7 @@
         <v>741</v>
       </c>
     </row>
-    <row r="189" spans="1:4">
+    <row r="189" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A189" t="s">
         <v>785</v>
       </c>
@@ -7994,7 +7999,7 @@
         <v>742</v>
       </c>
     </row>
-    <row r="190" spans="1:4">
+    <row r="190" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A190" t="s">
         <v>785</v>
       </c>
@@ -8008,7 +8013,7 @@
         <v>744</v>
       </c>
     </row>
-    <row r="191" spans="1:4">
+    <row r="191" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A191" t="s">
         <v>785</v>
       </c>
@@ -8022,7 +8027,7 @@
         <v>746</v>
       </c>
     </row>
-    <row r="192" spans="1:4">
+    <row r="192" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A192" t="s">
         <v>785</v>
       </c>
@@ -8036,7 +8041,7 @@
         <v>638</v>
       </c>
     </row>
-    <row r="193" spans="1:4">
+    <row r="193" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A193" t="s">
         <v>788</v>
       </c>
@@ -8050,7 +8055,7 @@
         <v>790</v>
       </c>
     </row>
-    <row r="194" spans="1:4">
+    <row r="194" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A194" t="s">
         <v>788</v>
       </c>
@@ -8064,7 +8069,7 @@
         <v>792</v>
       </c>
     </row>
-    <row r="195" spans="1:4">
+    <row r="195" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A195" t="s">
         <v>788</v>
       </c>
@@ -8078,7 +8083,7 @@
         <v>742</v>
       </c>
     </row>
-    <row r="196" spans="1:4">
+    <row r="196" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A196" t="s">
         <v>788</v>
       </c>
@@ -8092,7 +8097,7 @@
         <v>794</v>
       </c>
     </row>
-    <row r="197" spans="1:4">
+    <row r="197" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A197" t="s">
         <v>788</v>
       </c>
@@ -8106,7 +8111,7 @@
         <v>796</v>
       </c>
     </row>
-    <row r="198" spans="1:4">
+    <row r="198" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A198" t="s">
         <v>788</v>
       </c>
@@ -8128,9 +8133,9 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:B2"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
-    <row r="1" spans="1:2">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>797</v>
       </c>
@@ -8138,7 +8143,7 @@
         <v>798</v>
       </c>
     </row>
-    <row r="2" spans="1:2">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>799</v>
       </c>

</xml_diff>